<commit_message>
fix: fix BOM file (LED color)
Signed-off-by: T-Kimura-MM <tkc1110bs@gmail.com>
</commit_message>
<xml_diff>
--- a/MINI_VESC_PCBGoGo.xlsx
+++ b/MINI_VESC_PCBGoGo.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="238" uniqueCount="140">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="238" uniqueCount="141">
   <si>
     <t xml:space="preserve">品名
 Name</t>
@@ -258,6 +258,9 @@
   </si>
   <si>
     <t xml:space="preserve">D4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SML-P11UTT86R</t>
   </si>
   <si>
     <t xml:space="preserve">コネクタ</t>
@@ -769,9 +772,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>1</xdr:col>
-      <xdr:colOff>281160</xdr:colOff>
+      <xdr:colOff>280800</xdr:colOff>
       <xdr:row>0</xdr:row>
-      <xdr:rowOff>477360</xdr:rowOff>
+      <xdr:rowOff>477000</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -785,7 +788,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="142920" y="69840"/>
-          <a:ext cx="1293840" cy="407520"/>
+          <a:ext cx="1293480" cy="407160"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -806,7 +809,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:I37"/>
-  <sheetFormatPr defaultColWidth="9.03125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="9.0390625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="16.38"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="45.04"/>
@@ -1122,7 +1125,7 @@
         <v>42</v>
       </c>
       <c r="H12" s="5" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="I12" s="5" t="s">
         <v>39</v>
@@ -1130,26 +1133,26 @@
     </row>
     <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="5" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="C13" s="5" t="n">
         <v>1</v>
       </c>
       <c r="D13" s="5" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="E13" s="5" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="F13" s="5"/>
       <c r="G13" s="5" t="s">
+        <v>50</v>
+      </c>
+      <c r="H13" s="5" t="s">
         <v>49</v>
-      </c>
-      <c r="H13" s="5" t="s">
-        <v>48</v>
       </c>
       <c r="I13" s="5" t="s">
         <v>39</v>
@@ -1157,26 +1160,26 @@
     </row>
     <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="5" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="B14" s="5" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="C14" s="5" t="n">
         <v>1</v>
       </c>
       <c r="D14" s="5" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="E14" s="5" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="F14" s="5"/>
       <c r="G14" s="5" t="s">
+        <v>54</v>
+      </c>
+      <c r="H14" s="5" t="s">
         <v>53</v>
-      </c>
-      <c r="H14" s="5" t="s">
-        <v>52</v>
       </c>
       <c r="I14" s="5" t="s">
         <v>39</v>
@@ -1184,26 +1187,26 @@
     </row>
     <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="5" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="B15" s="5" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="C15" s="5" t="n">
         <v>1</v>
       </c>
       <c r="D15" s="5" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="E15" s="5" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="F15" s="5"/>
       <c r="G15" s="5" t="s">
+        <v>54</v>
+      </c>
+      <c r="H15" s="5" t="s">
         <v>53</v>
-      </c>
-      <c r="H15" s="5" t="s">
-        <v>52</v>
       </c>
       <c r="I15" s="5" t="s">
         <v>39</v>
@@ -1211,26 +1214,26 @@
     </row>
     <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="5" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="B16" s="5" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="C16" s="5" t="n">
         <v>1</v>
       </c>
       <c r="D16" s="5" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="E16" s="5" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="F16" s="5"/>
       <c r="G16" s="5" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="H16" s="5" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="I16" s="5" t="s">
         <v>39</v>
@@ -1238,23 +1241,23 @@
     </row>
     <row r="17" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="5" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="B17" s="5" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="C17" s="5" t="n">
         <v>1</v>
       </c>
       <c r="D17" s="5" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="E17" s="5" t="n">
         <v>3030</v>
       </c>
       <c r="F17" s="5"/>
       <c r="G17" s="5" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="H17" s="5" t="n">
         <v>74438335220</v>
@@ -1265,26 +1268,26 @@
     </row>
     <row r="18" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="5" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="B18" s="5" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="C18" s="5" t="n">
         <v>3</v>
       </c>
       <c r="D18" s="5" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="E18" s="5" t="n">
         <v>1608</v>
       </c>
       <c r="F18" s="5"/>
       <c r="G18" s="5" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="H18" s="5" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="I18" s="5" t="s">
         <v>39</v>
@@ -1292,26 +1295,26 @@
     </row>
     <row r="19" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="5" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="B19" s="5" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="C19" s="5" t="n">
         <v>3</v>
       </c>
       <c r="D19" s="5" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="E19" s="5" t="s">
         <v>20</v>
       </c>
       <c r="F19" s="5"/>
       <c r="G19" s="5" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="H19" s="5" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="I19" s="5" t="s">
         <v>14</v>
@@ -1319,26 +1322,26 @@
     </row>
     <row r="20" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="5" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="B20" s="5" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="C20" s="5" t="n">
         <v>4</v>
       </c>
       <c r="D20" s="5" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="E20" s="5" t="s">
         <v>20</v>
       </c>
       <c r="F20" s="5"/>
       <c r="G20" s="5" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="H20" s="5" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="I20" s="5" t="s">
         <v>14</v>
@@ -1346,10 +1349,10 @@
     </row>
     <row r="21" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="5" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="B21" s="5" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="C21" s="5" t="n">
         <v>3</v>
@@ -1362,10 +1365,10 @@
       </c>
       <c r="F21" s="5"/>
       <c r="G21" s="5" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="H21" s="5" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="I21" s="5" t="s">
         <v>14</v>
@@ -1373,26 +1376,26 @@
     </row>
     <row r="22" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="5" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="B22" s="5" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="C22" s="5" t="n">
         <v>3</v>
       </c>
       <c r="D22" s="5" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="E22" s="5" t="s">
         <v>20</v>
       </c>
       <c r="F22" s="5"/>
       <c r="G22" s="5" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="H22" s="5" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="I22" s="5" t="s">
         <v>14</v>
@@ -1400,26 +1403,26 @@
     </row>
     <row r="23" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="5" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="B23" s="5" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="C23" s="5" t="n">
         <v>1</v>
       </c>
       <c r="D23" s="5" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="E23" s="5" t="s">
         <v>20</v>
       </c>
       <c r="F23" s="5"/>
       <c r="G23" s="5" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="H23" s="5" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="I23" s="5" t="s">
         <v>14</v>
@@ -1427,26 +1430,26 @@
     </row>
     <row r="24" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="5" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="B24" s="5" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="C24" s="5" t="n">
         <v>3</v>
       </c>
       <c r="D24" s="5" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="E24" s="5" t="s">
         <v>20</v>
       </c>
       <c r="F24" s="5"/>
       <c r="G24" s="5" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="H24" s="5" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="I24" s="5" t="s">
         <v>14</v>
@@ -1454,26 +1457,26 @@
     </row>
     <row r="25" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="5" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="B25" s="5" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="C25" s="5" t="n">
         <v>2</v>
       </c>
       <c r="D25" s="5" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="E25" s="5" t="s">
         <v>20</v>
       </c>
       <c r="F25" s="5"/>
       <c r="G25" s="5" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="H25" s="5" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="I25" s="5" t="s">
         <v>14</v>
@@ -1481,26 +1484,26 @@
     </row>
     <row r="26" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="5" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="B26" s="5" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="C26" s="5" t="n">
         <v>1</v>
       </c>
       <c r="D26" s="5" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="E26" s="5" t="s">
         <v>20</v>
       </c>
       <c r="F26" s="5"/>
       <c r="G26" s="5" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="H26" s="5" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="I26" s="5" t="s">
         <v>14</v>
@@ -1508,26 +1511,26 @@
     </row>
     <row r="27" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="5" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="B27" s="5" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="C27" s="5" t="n">
         <v>1</v>
       </c>
       <c r="D27" s="5" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="E27" s="5" t="s">
         <v>20</v>
       </c>
       <c r="F27" s="5"/>
       <c r="G27" s="5" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="H27" s="5" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="I27" s="5" t="s">
         <v>14</v>
@@ -1535,26 +1538,26 @@
     </row>
     <row r="28" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="5" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="B28" s="5" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="C28" s="5" t="n">
         <v>1</v>
       </c>
       <c r="D28" s="5" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="E28" s="5" t="s">
         <v>20</v>
       </c>
       <c r="F28" s="5"/>
       <c r="G28" s="5" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="H28" s="5" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="I28" s="5" t="s">
         <v>14</v>
@@ -1562,26 +1565,26 @@
     </row>
     <row r="29" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="5" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="B29" s="6" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="C29" s="5" t="n">
         <v>3</v>
       </c>
       <c r="D29" s="5" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="E29" s="5" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="F29" s="5"/>
       <c r="G29" s="5" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="H29" s="5" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="I29" s="5" t="s">
         <v>39</v>
@@ -1589,26 +1592,26 @@
     </row>
     <row r="30" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="5" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="B30" s="5" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="C30" s="5" t="n">
         <v>3</v>
       </c>
       <c r="D30" s="5" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="E30" s="5" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="F30" s="5"/>
       <c r="G30" s="5" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="H30" s="5" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="I30" s="5" t="s">
         <v>39</v>
@@ -1616,26 +1619,26 @@
     </row>
     <row r="31" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="5" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="B31" s="5" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="C31" s="5" t="n">
         <v>1</v>
       </c>
       <c r="D31" s="5" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="E31" s="5" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="F31" s="5"/>
       <c r="G31" s="5" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="H31" s="5" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="I31" s="5" t="s">
         <v>39</v>
@@ -1643,26 +1646,26 @@
     </row>
     <row r="32" customFormat="false" ht="16.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="5" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="B32" s="5" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="C32" s="5" t="n">
         <v>1</v>
       </c>
       <c r="D32" s="5" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="E32" s="5" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="F32" s="5"/>
       <c r="G32" s="5" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="H32" s="5" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="I32" s="5" t="s">
         <v>39</v>
@@ -1670,26 +1673,26 @@
     </row>
     <row r="33" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="5" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="B33" s="5" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="C33" s="5" t="n">
         <v>2</v>
       </c>
       <c r="D33" s="5" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="E33" s="5" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="F33" s="5"/>
       <c r="G33" s="5" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="H33" s="5" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="I33" s="5" t="s">
         <v>39</v>
@@ -1697,26 +1700,26 @@
     </row>
     <row r="34" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="5" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="B34" s="5" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="C34" s="5" t="n">
         <v>3</v>
       </c>
       <c r="D34" s="5" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="E34" s="5" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="F34" s="5"/>
       <c r="G34" s="5" t="s">
         <v>42</v>
       </c>
       <c r="H34" s="5" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="I34" s="5" t="s">
         <v>39</v>
@@ -1724,26 +1727,26 @@
     </row>
     <row r="35" customFormat="false" ht="16.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="5" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="B35" s="5" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="C35" s="5" t="n">
         <v>1</v>
       </c>
       <c r="D35" s="5" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="E35" s="5" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="F35" s="5"/>
       <c r="G35" s="5" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="H35" s="5" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="I35" s="5" t="s">
         <v>39</v>
@@ -1751,26 +1754,26 @@
     </row>
     <row r="36" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="5" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="B36" s="5" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="C36" s="5" t="n">
         <v>1</v>
       </c>
       <c r="D36" s="5" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="E36" s="5" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="F36" s="5"/>
       <c r="G36" s="5" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="H36" s="5" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="I36" s="5" t="s">
         <v>39</v>

</xml_diff>